<commit_message>
feat(questions): import embedded lesson and unit figures
Exact source tree of locally verified commit 6e5f53c7b075f17ad82f849e00c8d0f89ef67d4a. Includes optional revision images, compatible XLSX templates, offline support and focused UI/PG17 verification.
</commit_message>
<xml_diff>
--- a/public/content-import-templates/09_official_book_questions_template.xlsx
+++ b/public/content-import-templates/09_official_book_questions_template.xlsx
@@ -753,20 +753,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B39"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac">
+  <dimension ref="A1:B42"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" ns2:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" s="1" customFormat="1" ns2:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ns2:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -774,7 +774,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ns2:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -782,7 +782,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ns2:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -790,12 +790,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" s="3" customFormat="1" ns2:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ns2:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -803,7 +803,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ns2:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -811,7 +811,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ns2:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -819,7 +819,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ns2:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -827,7 +827,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ns2:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -835,7 +835,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ns2:dyDescent="0.25">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -843,7 +843,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ns2:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -851,7 +851,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ns2:dyDescent="0.25">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -859,7 +859,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ns2:dyDescent="0.25">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -867,7 +867,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ns2:dyDescent="0.25">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -875,7 +875,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ns2:dyDescent="0.25">
       <c r="A18" t="s">
         <v>26</v>
       </c>
@@ -883,7 +883,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ns2:dyDescent="0.25">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -891,7 +891,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ns2:dyDescent="0.25">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -899,7 +899,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" ns2:dyDescent="0.25">
       <c r="A21" t="s">
         <v>29</v>
       </c>
@@ -907,7 +907,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" ns2:dyDescent="0.25">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -915,7 +915,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" ns2:dyDescent="0.25">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -923,7 +923,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ns2:dyDescent="0.25">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -931,7 +931,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" ns2:dyDescent="0.25">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -939,7 +939,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" ns2:dyDescent="0.25">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -947,12 +947,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" s="3" customFormat="1" ns2:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" ns2:dyDescent="0.25">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -960,7 +960,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" ns2:dyDescent="0.25">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -968,7 +968,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" ns2:dyDescent="0.25">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -976,7 +976,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" ns2:dyDescent="0.25">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -984,7 +984,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" ns2:dyDescent="0.25">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -992,7 +992,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" ns2:dyDescent="0.25">
       <c r="A34" t="s">
         <v>42</v>
       </c>
@@ -1000,7 +1000,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" ns2:dyDescent="0.25">
       <c r="A35" t="s">
         <v>42</v>
       </c>
@@ -1008,7 +1008,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" ns2:dyDescent="0.25">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" ns2:dyDescent="0.25">
       <c r="A37" t="s">
         <v>42</v>
       </c>
@@ -1024,7 +1024,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" ns2:dyDescent="0.25">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1032,12 +1032,36 @@
         <v>51</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" ns2:dyDescent="0.25">
       <c r="A39" t="s">
         <v>42</v>
       </c>
       <c r="B39" t="s">
         <v>52</v>
+      </c>
+    </row>
+    <row r="41" ht="74" customHeight="1">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>صورة السؤال (اختياري)</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>أدرج صورة PNG أو JPG فوق الخلايا وضع بدايتها في question_image بصف السؤال. اكتب وصفًا واضحًا في question_image_alt. صورة واحدة لكل سؤال، حتى 512 كيلوبايت.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="74" customHeight="1">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>إرشادات الصور</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>اترك قيمة خلية question_image فارغة. لا تستخدم روابط أو دالة IMAGE أو صور داخل الخلية. اترك العمودين فارغين إذا لم يتضمن السؤال صورة. تُرفع أسئلة الصور من استيراد محتويات الدرس.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1290,9 +1314,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac">
+  <dimension ref="A1:U2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" ns2:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -1307,9 +1331,11 @@
     <col min="17" max="17" width="19" customWidth="1"/>
     <col min="18" max="18" width="18" customWidth="1"/>
     <col min="19" max="19" width="21" customWidth="1"/>
+    <col min="20" max="20" width="28" customWidth="1"/>
+    <col min="21" max="21" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:19" s="4" customFormat="1" ns2:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>8</v>
       </c>
@@ -1367,8 +1393,18 @@
       <c r="S1" s="4" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>question_image</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>question_image_alt</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ns2:dyDescent="0.25">
       <c r="A2" t="s">
         <v>103</v>
       </c>
@@ -1428,7 +1464,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S1"/>
+  <autoFilter ref="A1:U2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(questions): support embedded lesson and unit images (#234)
* feat(questions): import embedded lesson and unit figures

Exact source tree of locally verified commit 6e5f53c7b075f17ad82f849e00c8d0f89ef67d4a. Includes optional revision images, compatible XLSX templates, offline support and focused UI/PG17 verification.

* test(questions): satisfy lint and record remote validation
</commit_message>
<xml_diff>
--- a/public/content-import-templates/09_official_book_questions_template.xlsx
+++ b/public/content-import-templates/09_official_book_questions_template.xlsx
@@ -753,20 +753,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B39"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac">
+  <dimension ref="A1:B42"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" ns2:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" s="1" customFormat="1" ns2:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ns2:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -774,7 +774,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ns2:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -782,7 +782,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ns2:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -790,12 +790,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" s="3" customFormat="1" ns2:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ns2:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -803,7 +803,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ns2:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -811,7 +811,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ns2:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -819,7 +819,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ns2:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -827,7 +827,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ns2:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -835,7 +835,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ns2:dyDescent="0.25">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -843,7 +843,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ns2:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -851,7 +851,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ns2:dyDescent="0.25">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -859,7 +859,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ns2:dyDescent="0.25">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -867,7 +867,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ns2:dyDescent="0.25">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -875,7 +875,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ns2:dyDescent="0.25">
       <c r="A18" t="s">
         <v>26</v>
       </c>
@@ -883,7 +883,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ns2:dyDescent="0.25">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -891,7 +891,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ns2:dyDescent="0.25">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -899,7 +899,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" ns2:dyDescent="0.25">
       <c r="A21" t="s">
         <v>29</v>
       </c>
@@ -907,7 +907,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" ns2:dyDescent="0.25">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -915,7 +915,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" ns2:dyDescent="0.25">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -923,7 +923,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ns2:dyDescent="0.25">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -931,7 +931,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" ns2:dyDescent="0.25">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -939,7 +939,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" ns2:dyDescent="0.25">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -947,12 +947,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" s="3" customFormat="1" ns2:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" ns2:dyDescent="0.25">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -960,7 +960,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" ns2:dyDescent="0.25">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -968,7 +968,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" ns2:dyDescent="0.25">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -976,7 +976,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" ns2:dyDescent="0.25">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -984,7 +984,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" ns2:dyDescent="0.25">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -992,7 +992,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" ns2:dyDescent="0.25">
       <c r="A34" t="s">
         <v>42</v>
       </c>
@@ -1000,7 +1000,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" ns2:dyDescent="0.25">
       <c r="A35" t="s">
         <v>42</v>
       </c>
@@ -1008,7 +1008,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" ns2:dyDescent="0.25">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" ns2:dyDescent="0.25">
       <c r="A37" t="s">
         <v>42</v>
       </c>
@@ -1024,7 +1024,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" ns2:dyDescent="0.25">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1032,12 +1032,36 @@
         <v>51</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" ns2:dyDescent="0.25">
       <c r="A39" t="s">
         <v>42</v>
       </c>
       <c r="B39" t="s">
         <v>52</v>
+      </c>
+    </row>
+    <row r="41" ht="74" customHeight="1">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>صورة السؤال (اختياري)</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>أدرج صورة PNG أو JPG فوق الخلايا وضع بدايتها في question_image بصف السؤال. اكتب وصفًا واضحًا في question_image_alt. صورة واحدة لكل سؤال، حتى 512 كيلوبايت.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="74" customHeight="1">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>إرشادات الصور</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>اترك قيمة خلية question_image فارغة. لا تستخدم روابط أو دالة IMAGE أو صور داخل الخلية. اترك العمودين فارغين إذا لم يتضمن السؤال صورة. تُرفع أسئلة الصور من استيراد محتويات الدرس.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1290,9 +1314,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac">
+  <dimension ref="A1:U2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" ns2:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -1307,9 +1331,11 @@
     <col min="17" max="17" width="19" customWidth="1"/>
     <col min="18" max="18" width="18" customWidth="1"/>
     <col min="19" max="19" width="21" customWidth="1"/>
+    <col min="20" max="20" width="28" customWidth="1"/>
+    <col min="21" max="21" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:19" s="4" customFormat="1" ns2:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>8</v>
       </c>
@@ -1367,8 +1393,18 @@
       <c r="S1" s="4" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>question_image</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>question_image_alt</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ns2:dyDescent="0.25">
       <c r="A2" t="s">
         <v>103</v>
       </c>
@@ -1428,7 +1464,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S1"/>
+  <autoFilter ref="A1:U2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>